<commit_message>
added method for gst customer add
</commit_message>
<xml_diff>
--- a/SoftwareRequirment.xlsx
+++ b/SoftwareRequirment.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27628"/>
+  <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Anjani\Project\AWS\iSoft\Tax_Managemnt\TaxConsultencyOfficeManagement\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Anjani\TaxConsultionOfficeManagement\TaxConsultingOfficeManagmement\ISoftTechSolutions\TaxConsultencyOfficeManagement\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B96F6783-14D9-4D25-A149-90E9DBF08661}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="12" activeTab="15"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="12" activeTab="15" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Plan" sheetId="12" r:id="rId1"/>
@@ -776,7 +777,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -937,7 +938,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -956,31 +957,7 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -993,25 +970,43 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="5" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="5" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="5" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1331,7 +1326,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B5"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -1375,7 +1370,7 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
   <dimension ref="A1:D14"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -1384,18 +1379,18 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="B1" s="12"/>
-      <c r="C1" s="12"/>
-      <c r="D1" s="12"/>
+      <c r="B1" s="15"/>
+      <c r="C1" s="15"/>
+      <c r="D1" s="15"/>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A2" s="12"/>
-      <c r="B2" s="12"/>
-      <c r="C2" s="12"/>
-      <c r="D2" s="12"/>
+      <c r="A2" s="15"/>
+      <c r="B2" s="15"/>
+      <c r="C2" s="15"/>
+      <c r="D2" s="15"/>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
@@ -1472,7 +1467,7 @@
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
   <dimension ref="A1:A11"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -1540,7 +1535,7 @@
 </file>
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0B00-000000000000}">
   <dimension ref="A1:A3"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -1568,7 +1563,7 @@
 </file>
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0C00-000000000000}">
   <dimension ref="A1:A9"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -1626,7 +1621,7 @@
 </file>
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0D00-000000000000}">
   <dimension ref="A1:A2"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -1649,7 +1644,7 @@
 </file>
 
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0E00-000000000000}">
   <dimension ref="A1:F4"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -1702,264 +1697,264 @@
 </file>
 
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0F00-000000000000}">
   <dimension ref="C1:F41"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="3" max="3" width="19.81640625" customWidth="1"/>
-    <col min="4" max="4" width="22.81640625" style="20" customWidth="1"/>
-    <col min="5" max="5" width="38.54296875" style="18" customWidth="1"/>
-    <col min="6" max="6" width="42.26953125" style="20" customWidth="1"/>
+    <col min="4" max="4" width="22.81640625" style="12" customWidth="1"/>
+    <col min="5" max="5" width="38.54296875" style="10" customWidth="1"/>
+    <col min="6" max="6" width="42.26953125" style="12" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="3:6" x14ac:dyDescent="0.35">
-      <c r="C1" s="22" t="s">
+      <c r="C1" s="19" t="s">
         <v>210</v>
       </c>
-      <c r="D1" s="16"/>
-      <c r="E1" s="16"/>
-      <c r="F1" s="16"/>
+      <c r="D1" s="20"/>
+      <c r="E1" s="20"/>
+      <c r="F1" s="20"/>
     </row>
     <row r="2" spans="3:6" x14ac:dyDescent="0.35">
-      <c r="C2" s="16"/>
-      <c r="D2" s="16"/>
-      <c r="E2" s="16"/>
-      <c r="F2" s="16"/>
+      <c r="C2" s="20"/>
+      <c r="D2" s="20"/>
+      <c r="E2" s="20"/>
+      <c r="F2" s="20"/>
     </row>
     <row r="3" spans="3:6" x14ac:dyDescent="0.35">
-      <c r="C3" s="23" t="s">
+      <c r="C3" s="21" t="s">
         <v>112</v>
       </c>
-      <c r="D3" s="24" t="s">
+      <c r="D3" s="23" t="s">
         <v>113</v>
       </c>
       <c r="E3" s="25" t="s">
         <v>114</v>
       </c>
-      <c r="F3" s="24" t="s">
+      <c r="F3" s="23" t="s">
         <v>115</v>
       </c>
     </row>
     <row r="4" spans="3:6" x14ac:dyDescent="0.35">
-      <c r="C4" s="26"/>
-      <c r="D4" s="27"/>
-      <c r="E4" s="28"/>
-      <c r="F4" s="27"/>
+      <c r="C4" s="22"/>
+      <c r="D4" s="24"/>
+      <c r="E4" s="26"/>
+      <c r="F4" s="24"/>
     </row>
     <row r="5" spans="3:6" ht="29" x14ac:dyDescent="0.35">
-      <c r="C5" s="13" t="s">
+      <c r="C5" s="8" t="s">
         <v>116</v>
       </c>
-      <c r="D5" s="19" t="s">
+      <c r="D5" s="11" t="s">
         <v>117</v>
       </c>
-      <c r="E5" s="17" t="s">
+      <c r="E5" s="9" t="s">
         <v>118</v>
       </c>
-      <c r="F5" s="19" t="s">
+      <c r="F5" s="11" t="s">
         <v>119</v>
       </c>
     </row>
     <row r="6" spans="3:6" ht="29" x14ac:dyDescent="0.35">
-      <c r="C6" s="14" t="s">
+      <c r="C6" s="16" t="s">
         <v>120</v>
       </c>
-      <c r="D6" s="19" t="s">
+      <c r="D6" s="11" t="s">
         <v>121</v>
       </c>
-      <c r="E6" s="17" t="s">
+      <c r="E6" s="9" t="s">
         <v>122</v>
       </c>
-      <c r="F6" s="19" t="s">
+      <c r="F6" s="11" t="s">
         <v>123</v>
       </c>
     </row>
     <row r="7" spans="3:6" ht="29" x14ac:dyDescent="0.35">
-      <c r="C7" s="15"/>
-      <c r="D7" s="19" t="s">
+      <c r="C7" s="18"/>
+      <c r="D7" s="11" t="s">
         <v>124</v>
       </c>
-      <c r="E7" s="17" t="s">
+      <c r="E7" s="9" t="s">
         <v>125</v>
       </c>
-      <c r="F7" s="19" t="s">
+      <c r="F7" s="11" t="s">
         <v>126</v>
       </c>
     </row>
     <row r="8" spans="3:6" ht="29" x14ac:dyDescent="0.35">
-      <c r="C8" s="14" t="s">
+      <c r="C8" s="16" t="s">
         <v>127</v>
       </c>
-      <c r="D8" s="19" t="s">
+      <c r="D8" s="11" t="s">
         <v>128</v>
       </c>
-      <c r="E8" s="17" t="s">
+      <c r="E8" s="9" t="s">
         <v>129</v>
       </c>
-      <c r="F8" s="19" t="s">
+      <c r="F8" s="11" t="s">
         <v>130</v>
       </c>
     </row>
     <row r="9" spans="3:6" ht="29" x14ac:dyDescent="0.35">
-      <c r="C9" s="15"/>
-      <c r="D9" s="19" t="s">
+      <c r="C9" s="18"/>
+      <c r="D9" s="11" t="s">
         <v>131</v>
       </c>
-      <c r="E9" s="17" t="s">
+      <c r="E9" s="9" t="s">
         <v>132</v>
       </c>
-      <c r="F9" s="19" t="s">
+      <c r="F9" s="11" t="s">
         <v>133</v>
       </c>
     </row>
     <row r="10" spans="3:6" ht="29" x14ac:dyDescent="0.35">
-      <c r="C10" s="14" t="s">
+      <c r="C10" s="16" t="s">
         <v>134</v>
       </c>
-      <c r="D10" s="19" t="s">
+      <c r="D10" s="11" t="s">
         <v>135</v>
       </c>
-      <c r="E10" s="17" t="s">
+      <c r="E10" s="9" t="s">
         <v>136</v>
       </c>
-      <c r="F10" s="19" t="s">
+      <c r="F10" s="11" t="s">
         <v>137</v>
       </c>
     </row>
     <row r="11" spans="3:6" ht="29" x14ac:dyDescent="0.35">
-      <c r="C11" s="21"/>
-      <c r="D11" s="19" t="s">
+      <c r="C11" s="17"/>
+      <c r="D11" s="11" t="s">
         <v>138</v>
       </c>
-      <c r="E11" s="17" t="s">
+      <c r="E11" s="9" t="s">
         <v>139</v>
       </c>
-      <c r="F11" s="19" t="s">
+      <c r="F11" s="11" t="s">
         <v>140</v>
       </c>
     </row>
     <row r="12" spans="3:6" ht="29" x14ac:dyDescent="0.35">
-      <c r="C12" s="15"/>
-      <c r="D12" s="19" t="s">
+      <c r="C12" s="18"/>
+      <c r="D12" s="11" t="s">
         <v>141</v>
       </c>
-      <c r="E12" s="17" t="s">
+      <c r="E12" s="9" t="s">
         <v>142</v>
       </c>
-      <c r="F12" s="19" t="s">
+      <c r="F12" s="11" t="s">
         <v>143</v>
       </c>
     </row>
     <row r="13" spans="3:6" ht="29" x14ac:dyDescent="0.35">
-      <c r="C13" s="14" t="s">
+      <c r="C13" s="16" t="s">
         <v>144</v>
       </c>
-      <c r="D13" s="19" t="s">
+      <c r="D13" s="11" t="s">
         <v>145</v>
       </c>
-      <c r="E13" s="17" t="s">
+      <c r="E13" s="9" t="s">
         <v>146</v>
       </c>
-      <c r="F13" s="19" t="s">
+      <c r="F13" s="11" t="s">
         <v>147</v>
       </c>
     </row>
     <row r="14" spans="3:6" ht="29" x14ac:dyDescent="0.35">
-      <c r="C14" s="21"/>
-      <c r="D14" s="19" t="s">
+      <c r="C14" s="17"/>
+      <c r="D14" s="11" t="s">
         <v>148</v>
       </c>
-      <c r="E14" s="17" t="s">
+      <c r="E14" s="9" t="s">
         <v>149</v>
       </c>
-      <c r="F14" s="19" t="s">
+      <c r="F14" s="11" t="s">
         <v>150</v>
       </c>
     </row>
     <row r="15" spans="3:6" x14ac:dyDescent="0.35">
-      <c r="C15" s="15"/>
-      <c r="D15" s="20" t="s">
+      <c r="C15" s="18"/>
+      <c r="D15" s="12" t="s">
         <v>151</v>
       </c>
-      <c r="E15" s="17" t="s">
+      <c r="E15" s="9" t="s">
         <v>152</v>
       </c>
-      <c r="F15" s="19" t="s">
+      <c r="F15" s="11" t="s">
         <v>153</v>
       </c>
     </row>
     <row r="16" spans="3:6" ht="29" x14ac:dyDescent="0.35">
-      <c r="C16" s="14" t="s">
+      <c r="C16" s="16" t="s">
         <v>154</v>
       </c>
-      <c r="D16" s="20" t="s">
+      <c r="D16" s="12" t="s">
         <v>155</v>
       </c>
-      <c r="E16" s="17" t="s">
+      <c r="E16" s="9" t="s">
         <v>156</v>
       </c>
-      <c r="F16" s="19" t="s">
+      <c r="F16" s="11" t="s">
         <v>157</v>
       </c>
     </row>
     <row r="17" spans="3:6" x14ac:dyDescent="0.35">
-      <c r="C17" s="15"/>
-      <c r="D17" s="20" t="s">
+      <c r="C17" s="18"/>
+      <c r="D17" s="12" t="s">
         <v>158</v>
       </c>
-      <c r="E17" s="17" t="s">
+      <c r="E17" s="9" t="s">
         <v>159</v>
       </c>
-      <c r="F17" s="19" t="s">
+      <c r="F17" s="11" t="s">
         <v>160</v>
       </c>
     </row>
     <row r="18" spans="3:6" ht="29" x14ac:dyDescent="0.35">
-      <c r="C18" s="14" t="s">
+      <c r="C18" s="16" t="s">
         <v>161</v>
       </c>
-      <c r="D18" s="20" t="s">
+      <c r="D18" s="12" t="s">
         <v>162</v>
       </c>
-      <c r="E18" s="17" t="s">
+      <c r="E18" s="9" t="s">
         <v>163</v>
       </c>
-      <c r="F18" s="19" t="s">
+      <c r="F18" s="11" t="s">
         <v>164</v>
       </c>
     </row>
     <row r="19" spans="3:6" ht="29" x14ac:dyDescent="0.35">
-      <c r="C19" s="21"/>
-      <c r="D19" s="20" t="s">
+      <c r="C19" s="17"/>
+      <c r="D19" s="12" t="s">
         <v>165</v>
       </c>
-      <c r="E19" s="17" t="s">
+      <c r="E19" s="9" t="s">
         <v>166</v>
       </c>
-      <c r="F19" s="19" t="s">
+      <c r="F19" s="11" t="s">
         <v>167</v>
       </c>
     </row>
     <row r="20" spans="3:6" x14ac:dyDescent="0.35">
-      <c r="C20" s="15"/>
-      <c r="D20" s="20" t="s">
+      <c r="C20" s="18"/>
+      <c r="D20" s="12" t="s">
         <v>168</v>
       </c>
-      <c r="E20" s="17" t="s">
+      <c r="E20" s="9" t="s">
         <v>169</v>
       </c>
-      <c r="F20" s="19" t="s">
+      <c r="F20" s="11" t="s">
         <v>170</v>
       </c>
     </row>
     <row r="21" spans="3:6" x14ac:dyDescent="0.35">
-      <c r="C21" s="14" t="s">
+      <c r="C21" s="16" t="s">
         <v>171</v>
       </c>
-      <c r="D21" s="20" t="s">
+      <c r="D21" s="12" t="s">
         <v>172</v>
       </c>
-      <c r="E21" s="20" t="s">
+      <c r="E21" s="12" t="s">
         <v>173</v>
       </c>
       <c r="F21" t="s">
@@ -1967,23 +1962,23 @@
       </c>
     </row>
     <row r="22" spans="3:6" x14ac:dyDescent="0.35">
-      <c r="C22" s="21"/>
-      <c r="D22" s="19" t="s">
+      <c r="C22" s="17"/>
+      <c r="D22" s="11" t="s">
         <v>175</v>
       </c>
-      <c r="E22" s="20" t="s">
+      <c r="E22" s="12" t="s">
         <v>176</v>
       </c>
-      <c r="F22" s="19" t="s">
+      <c r="F22" s="11" t="s">
         <v>177</v>
       </c>
     </row>
     <row r="23" spans="3:6" x14ac:dyDescent="0.35">
-      <c r="C23" s="21"/>
-      <c r="D23" s="19" t="s">
+      <c r="C23" s="17"/>
+      <c r="D23" s="11" t="s">
         <v>178</v>
       </c>
-      <c r="E23" s="20" t="s">
+      <c r="E23" s="12" t="s">
         <v>179</v>
       </c>
       <c r="F23" t="s">
@@ -1991,225 +1986,215 @@
       </c>
     </row>
     <row r="24" spans="3:6" x14ac:dyDescent="0.35">
-      <c r="C24" s="15"/>
-      <c r="D24" s="19" t="s">
+      <c r="C24" s="18"/>
+      <c r="D24" s="11" t="s">
         <v>181</v>
       </c>
-      <c r="E24" s="20" t="s">
+      <c r="E24" s="12" t="s">
         <v>182</v>
       </c>
-      <c r="F24" s="19" t="s">
+      <c r="F24" s="11" t="s">
         <v>183</v>
       </c>
     </row>
     <row r="25" spans="3:6" ht="29" x14ac:dyDescent="0.35">
-      <c r="C25" s="14" t="s">
+      <c r="C25" s="16" t="s">
         <v>184</v>
       </c>
-      <c r="D25" s="20" t="s">
+      <c r="D25" s="12" t="s">
         <v>185</v>
       </c>
-      <c r="E25" s="20" t="s">
+      <c r="E25" s="12" t="s">
         <v>186</v>
       </c>
-      <c r="F25" s="19" t="s">
+      <c r="F25" s="11" t="s">
         <v>187</v>
       </c>
     </row>
     <row r="26" spans="3:6" ht="29" x14ac:dyDescent="0.35">
-      <c r="C26" s="21"/>
-      <c r="D26" s="19" t="s">
+      <c r="C26" s="17"/>
+      <c r="D26" s="11" t="s">
         <v>188</v>
       </c>
-      <c r="E26" s="20" t="s">
+      <c r="E26" s="12" t="s">
         <v>189</v>
       </c>
-      <c r="F26" s="19" t="s">
+      <c r="F26" s="11" t="s">
         <v>190</v>
       </c>
     </row>
     <row r="27" spans="3:6" ht="29" x14ac:dyDescent="0.35">
-      <c r="C27" s="15"/>
-      <c r="D27" s="19" t="s">
+      <c r="C27" s="18"/>
+      <c r="D27" s="11" t="s">
         <v>191</v>
       </c>
-      <c r="E27" s="20" t="s">
+      <c r="E27" s="12" t="s">
         <v>192</v>
       </c>
-      <c r="F27" s="19" t="s">
+      <c r="F27" s="11" t="s">
         <v>193</v>
       </c>
     </row>
     <row r="28" spans="3:6" ht="29" x14ac:dyDescent="0.35">
-      <c r="C28" s="14" t="s">
+      <c r="C28" s="16" t="s">
         <v>194</v>
       </c>
-      <c r="D28" s="19" t="s">
+      <c r="D28" s="11" t="s">
         <v>195</v>
       </c>
-      <c r="E28" s="20" t="s">
+      <c r="E28" s="12" t="s">
         <v>196</v>
       </c>
-      <c r="F28" s="19" t="s">
+      <c r="F28" s="11" t="s">
         <v>197</v>
       </c>
     </row>
     <row r="29" spans="3:6" ht="29" x14ac:dyDescent="0.35">
-      <c r="C29" s="15"/>
-      <c r="D29" s="19" t="s">
+      <c r="C29" s="18"/>
+      <c r="D29" s="11" t="s">
         <v>198</v>
       </c>
-      <c r="E29" s="20" t="s">
+      <c r="E29" s="12" t="s">
         <v>196</v>
       </c>
-      <c r="F29" s="19" t="s">
+      <c r="F29" s="11" t="s">
         <v>199</v>
       </c>
     </row>
     <row r="30" spans="3:6" ht="29" x14ac:dyDescent="0.35">
-      <c r="C30" s="14" t="s">
+      <c r="C30" s="16" t="s">
         <v>200</v>
       </c>
-      <c r="D30" s="19" t="s">
+      <c r="D30" s="11" t="s">
         <v>201</v>
       </c>
-      <c r="E30" s="20" t="s">
+      <c r="E30" s="12" t="s">
         <v>202</v>
       </c>
-      <c r="F30" s="19" t="s">
+      <c r="F30" s="11" t="s">
         <v>203</v>
       </c>
     </row>
     <row r="31" spans="3:6" ht="29" x14ac:dyDescent="0.35">
-      <c r="C31" s="21"/>
-      <c r="D31" s="19" t="s">
+      <c r="C31" s="17"/>
+      <c r="D31" s="11" t="s">
         <v>204</v>
       </c>
-      <c r="E31" s="20" t="s">
+      <c r="E31" s="12" t="s">
         <v>205</v>
       </c>
-      <c r="F31" s="19" t="s">
+      <c r="F31" s="11" t="s">
         <v>206</v>
       </c>
     </row>
     <row r="32" spans="3:6" x14ac:dyDescent="0.35">
-      <c r="C32" s="15"/>
-      <c r="D32" s="19" t="s">
+      <c r="C32" s="18"/>
+      <c r="D32" s="11" t="s">
         <v>207</v>
       </c>
-      <c r="E32" s="20" t="s">
+      <c r="E32" s="12" t="s">
         <v>208</v>
       </c>
-      <c r="F32" s="19" t="s">
+      <c r="F32" s="11" t="s">
         <v>209</v>
       </c>
     </row>
     <row r="33" spans="3:6" x14ac:dyDescent="0.35">
-      <c r="C33" s="14" t="s">
+      <c r="C33" s="16" t="s">
         <v>211</v>
       </c>
-      <c r="D33" s="19" t="s">
+      <c r="D33" s="11" t="s">
         <v>212</v>
       </c>
-      <c r="E33" s="20" t="s">
+      <c r="E33" s="12" t="s">
         <v>213</v>
       </c>
-      <c r="F33" s="19" t="s">
+      <c r="F33" s="11" t="s">
         <v>214</v>
       </c>
     </row>
     <row r="34" spans="3:6" ht="29" x14ac:dyDescent="0.35">
-      <c r="C34" s="21"/>
-      <c r="D34" s="19" t="s">
+      <c r="C34" s="17"/>
+      <c r="D34" s="11" t="s">
         <v>215</v>
       </c>
-      <c r="E34" s="20" t="s">
+      <c r="E34" s="12" t="s">
         <v>216</v>
       </c>
-      <c r="F34" s="19" t="s">
+      <c r="F34" s="11" t="s">
         <v>217</v>
       </c>
     </row>
     <row r="35" spans="3:6" ht="29" x14ac:dyDescent="0.35">
-      <c r="C35" s="15"/>
-      <c r="D35" s="19" t="s">
+      <c r="C35" s="18"/>
+      <c r="D35" s="11" t="s">
         <v>218</v>
       </c>
-      <c r="E35" s="20" t="s">
+      <c r="E35" s="12" t="s">
         <v>219</v>
       </c>
-      <c r="F35" s="19" t="s">
+      <c r="F35" s="11" t="s">
         <v>220</v>
       </c>
     </row>
     <row r="36" spans="3:6" ht="29" x14ac:dyDescent="0.35">
-      <c r="C36" s="14" t="s">
+      <c r="C36" s="16" t="s">
         <v>221</v>
       </c>
-      <c r="D36" s="19" t="s">
+      <c r="D36" s="11" t="s">
         <v>222</v>
       </c>
-      <c r="E36" s="20" t="s">
+      <c r="E36" s="12" t="s">
         <v>223</v>
       </c>
-      <c r="F36" s="19" t="s">
+      <c r="F36" s="11" t="s">
         <v>224</v>
       </c>
     </row>
     <row r="37" spans="3:6" ht="29" x14ac:dyDescent="0.35">
-      <c r="C37" s="21"/>
-      <c r="D37" s="19" t="s">
+      <c r="C37" s="17"/>
+      <c r="D37" s="11" t="s">
         <v>225</v>
       </c>
-      <c r="E37" s="20" t="s">
+      <c r="E37" s="12" t="s">
         <v>226</v>
       </c>
-      <c r="F37" s="19" t="s">
+      <c r="F37" s="11" t="s">
         <v>227</v>
       </c>
     </row>
     <row r="38" spans="3:6" ht="29" x14ac:dyDescent="0.35">
-      <c r="C38" s="15"/>
-      <c r="D38" s="19" t="s">
+      <c r="C38" s="18"/>
+      <c r="D38" s="11" t="s">
         <v>228</v>
       </c>
-      <c r="E38" s="20" t="s">
+      <c r="E38" s="12" t="s">
         <v>229</v>
       </c>
-      <c r="F38" s="19" t="s">
+      <c r="F38" s="11" t="s">
         <v>230</v>
       </c>
     </row>
     <row r="39" spans="3:6" x14ac:dyDescent="0.35">
-      <c r="C39" s="13"/>
-      <c r="D39" s="19"/>
-      <c r="E39" s="17"/>
-      <c r="F39" s="19"/>
+      <c r="C39" s="8"/>
+      <c r="D39" s="11"/>
+      <c r="E39" s="9"/>
+      <c r="F39" s="11"/>
     </row>
     <row r="40" spans="3:6" x14ac:dyDescent="0.35">
-      <c r="C40" s="13"/>
-      <c r="D40" s="19"/>
-      <c r="E40" s="17"/>
-      <c r="F40" s="19"/>
+      <c r="C40" s="8"/>
+      <c r="D40" s="11"/>
+      <c r="E40" s="9"/>
+      <c r="F40" s="11"/>
     </row>
     <row r="41" spans="3:6" x14ac:dyDescent="0.35">
-      <c r="C41" s="13"/>
-      <c r="D41" s="19"/>
-      <c r="E41" s="17"/>
-      <c r="F41" s="19"/>
+      <c r="C41" s="8"/>
+      <c r="D41" s="11"/>
+      <c r="E41" s="9"/>
+      <c r="F41" s="11"/>
     </row>
   </sheetData>
   <mergeCells count="17">
-    <mergeCell ref="C25:C27"/>
-    <mergeCell ref="C28:C29"/>
-    <mergeCell ref="C30:C32"/>
-    <mergeCell ref="C33:C35"/>
-    <mergeCell ref="C36:C38"/>
-    <mergeCell ref="C8:C9"/>
-    <mergeCell ref="C10:C12"/>
-    <mergeCell ref="C13:C15"/>
-    <mergeCell ref="C16:C17"/>
-    <mergeCell ref="C18:C20"/>
     <mergeCell ref="C21:C24"/>
     <mergeCell ref="C1:F2"/>
     <mergeCell ref="C3:C4"/>
@@ -2217,6 +2202,16 @@
     <mergeCell ref="E3:E4"/>
     <mergeCell ref="F3:F4"/>
     <mergeCell ref="C6:C7"/>
+    <mergeCell ref="C8:C9"/>
+    <mergeCell ref="C10:C12"/>
+    <mergeCell ref="C13:C15"/>
+    <mergeCell ref="C16:C17"/>
+    <mergeCell ref="C18:C20"/>
+    <mergeCell ref="C25:C27"/>
+    <mergeCell ref="C28:C29"/>
+    <mergeCell ref="C30:C32"/>
+    <mergeCell ref="C33:C35"/>
+    <mergeCell ref="C36:C38"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -2224,7 +2219,7 @@
 </file>
 
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1000-000000000000}">
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData/>
@@ -2233,7 +2228,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:B10"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -2321,7 +2316,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:H14"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -2331,23 +2326,23 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="14.4" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="10" t="s">
+      <c r="A1" s="13" t="s">
         <v>93</v>
       </c>
-      <c r="B1" s="10"/>
-      <c r="C1" s="10"/>
+      <c r="B1" s="13"/>
+      <c r="C1" s="13"/>
       <c r="D1" s="7"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A2" s="10"/>
-      <c r="B2" s="10"/>
-      <c r="C2" s="10"/>
+      <c r="A2" s="13"/>
+      <c r="B2" s="13"/>
+      <c r="C2" s="13"/>
       <c r="D2" s="7"/>
     </row>
     <row r="3" spans="1:8" ht="36.65" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="11"/>
-      <c r="B3" s="11"/>
-      <c r="C3" s="11"/>
+      <c r="A3" s="14"/>
+      <c r="B3" s="14"/>
+      <c r="C3" s="14"/>
       <c r="D3" s="7"/>
     </row>
     <row r="4" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.35">
@@ -2421,10 +2416,10 @@
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A9" s="8" t="s">
+      <c r="A9" s="6" t="s">
         <v>109</v>
       </c>
-      <c r="B9" s="9" t="s">
+      <c r="B9" s="5" t="s">
         <v>110</v>
       </c>
       <c r="C9" t="s">
@@ -2443,7 +2438,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData/>
@@ -2452,7 +2447,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:D10"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -2460,24 +2455,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="15" t="s">
         <v>20</v>
       </c>
-      <c r="B1" s="12"/>
-      <c r="C1" s="12"/>
-      <c r="D1" s="12"/>
+      <c r="B1" s="15"/>
+      <c r="C1" s="15"/>
+      <c r="D1" s="15"/>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A2" s="12"/>
-      <c r="B2" s="12"/>
-      <c r="C2" s="12"/>
-      <c r="D2" s="12"/>
+      <c r="A2" s="15"/>
+      <c r="B2" s="15"/>
+      <c r="C2" s="15"/>
+      <c r="D2" s="15"/>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A3" s="12"/>
-      <c r="B3" s="12"/>
-      <c r="C3" s="12"/>
-      <c r="D3" s="12"/>
+      <c r="A3" s="15"/>
+      <c r="B3" s="15"/>
+      <c r="C3" s="15"/>
+      <c r="D3" s="15"/>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
@@ -2523,7 +2518,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:C5"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -2531,16 +2526,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="15" t="s">
         <v>34</v>
       </c>
-      <c r="B1" s="12"/>
-      <c r="C1" s="12"/>
+      <c r="B1" s="15"/>
+      <c r="C1" s="15"/>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A2" s="12"/>
-      <c r="B2" s="12"/>
-      <c r="C2" s="12"/>
+      <c r="A2" s="15"/>
+      <c r="B2" s="15"/>
+      <c r="C2" s="15"/>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
@@ -2566,7 +2561,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:D11"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -2574,24 +2569,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="15" t="s">
         <v>21</v>
       </c>
-      <c r="B1" s="12"/>
-      <c r="C1" s="12"/>
-      <c r="D1" s="12"/>
+      <c r="B1" s="15"/>
+      <c r="C1" s="15"/>
+      <c r="D1" s="15"/>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A2" s="12"/>
-      <c r="B2" s="12"/>
-      <c r="C2" s="12"/>
-      <c r="D2" s="12"/>
+      <c r="A2" s="15"/>
+      <c r="B2" s="15"/>
+      <c r="C2" s="15"/>
+      <c r="D2" s="15"/>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A3" s="12"/>
-      <c r="B3" s="12"/>
-      <c r="C3" s="12"/>
-      <c r="D3" s="12"/>
+      <c r="A3" s="15"/>
+      <c r="B3" s="15"/>
+      <c r="C3" s="15"/>
+      <c r="D3" s="15"/>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
@@ -2642,7 +2637,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <dimension ref="A1:D11"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -2651,24 +2646,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="15" t="s">
         <v>10</v>
       </c>
-      <c r="B1" s="12"/>
-      <c r="C1" s="12"/>
-      <c r="D1" s="12"/>
+      <c r="B1" s="15"/>
+      <c r="C1" s="15"/>
+      <c r="D1" s="15"/>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A2" s="12"/>
-      <c r="B2" s="12"/>
-      <c r="C2" s="12"/>
-      <c r="D2" s="12"/>
+      <c r="A2" s="15"/>
+      <c r="B2" s="15"/>
+      <c r="C2" s="15"/>
+      <c r="D2" s="15"/>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A3" s="12"/>
-      <c r="B3" s="12"/>
-      <c r="C3" s="12"/>
-      <c r="D3" s="12"/>
+      <c r="A3" s="15"/>
+      <c r="B3" s="15"/>
+      <c r="C3" s="15"/>
+      <c r="D3" s="15"/>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
@@ -2722,7 +2717,7 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
   <dimension ref="A1:D6"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -2730,18 +2725,18 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="15" t="s">
         <v>49</v>
       </c>
-      <c r="B1" s="12"/>
-      <c r="C1" s="12"/>
-      <c r="D1" s="12"/>
+      <c r="B1" s="15"/>
+      <c r="C1" s="15"/>
+      <c r="D1" s="15"/>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A2" s="12"/>
-      <c r="B2" s="12"/>
-      <c r="C2" s="12"/>
-      <c r="D2" s="12"/>
+      <c r="A2" s="15"/>
+      <c r="B2" s="15"/>
+      <c r="C2" s="15"/>
+      <c r="D2" s="15"/>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" t="s">

</xml_diff>

<commit_message>
Second Level Cache Implemeted for TdsCustomer
</commit_message>
<xml_diff>
--- a/SoftwareRequirment.xlsx
+++ b/SoftwareRequirment.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27726"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Anjani\TaxConsultionOfficeManagement\TaxConsultingOfficeManagmement\ISoftTechSolutions\TaxConsultencyOfficeManagement\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B96F6783-14D9-4D25-A149-90E9DBF08661}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{022219C0-CFF3-442E-9AE9-88317736B173}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="12" activeTab="15" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="12" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Plan" sheetId="12" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="245" uniqueCount="231">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="262" uniqueCount="247">
   <si>
     <t>Name</t>
   </si>
@@ -772,6 +772,54 @@
   </si>
   <si>
     <t>Easy setup, Docker support, parallel job execution</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Revnue Management </t>
+  </si>
+  <si>
+    <t>Rate Management</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Laoyalty Programe </t>
+  </si>
+  <si>
+    <t>Collection Managemnt</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Customer based on Type </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Filing by customer </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Revnue based on Customer </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Revnue based on Organization </t>
+  </si>
+  <si>
+    <t>TDS/GST filed based on Employee</t>
+  </si>
+  <si>
+    <t>TDS/GST filed based on Per month per year</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TDS/ GST filed based on Time Duration </t>
+  </si>
+  <si>
+    <t>Planning Fetheres</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S.No </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fethers </t>
+  </si>
+  <si>
+    <t>In Progress Fethers</t>
+  </si>
+  <si>
+    <t>Feathers</t>
   </si>
 </sst>
 </file>
@@ -938,7 +986,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1011,6 +1059,18 @@
     </xf>
     <xf numFmtId="49" fontId="5" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1564,58 +1624,158 @@
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0C00-000000000000}">
-  <dimension ref="A1:A9"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="44.81640625" customWidth="1"/>
+    <col min="2" max="2" width="44.81640625" customWidth="1"/>
+    <col min="5" max="5" width="43.54296875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A1" t="s">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A1" s="15" t="s">
+        <v>245</v>
+      </c>
+      <c r="B1" s="15"/>
+      <c r="D1" s="29" t="s">
+        <v>242</v>
+      </c>
+      <c r="E1" s="29"/>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A2" s="27"/>
+      <c r="B2" s="27"/>
+      <c r="D2" s="28"/>
+      <c r="E2" s="28"/>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A3" s="30" t="s">
+        <v>243</v>
+      </c>
+      <c r="B3" s="30" t="s">
+        <v>246</v>
+      </c>
+      <c r="D3" s="8" t="s">
+        <v>243</v>
+      </c>
+      <c r="E3" s="8" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A4" s="8"/>
+      <c r="B4" s="8" t="s">
         <v>69</v>
       </c>
-    </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
+      <c r="D4" s="8"/>
+      <c r="E4" s="8" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A5" s="8"/>
+      <c r="B5" s="8" t="s">
         <v>68</v>
       </c>
-    </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A3" t="s">
+      <c r="D5" s="8"/>
+      <c r="E5" s="8" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A6" s="8"/>
+      <c r="B6" s="8" t="s">
         <v>70</v>
       </c>
-    </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A4" t="s">
+      <c r="D6" s="8"/>
+      <c r="E6" s="8" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A7" s="8"/>
+      <c r="B7" s="8" t="s">
         <v>63</v>
       </c>
-    </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A5" t="s">
+      <c r="D7" s="8"/>
+      <c r="E7" s="8" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A8" s="8"/>
+      <c r="B8" s="8" t="s">
         <v>64</v>
       </c>
-    </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A6" t="s">
+      <c r="D8" s="8"/>
+      <c r="E8" s="8" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A9" s="8"/>
+      <c r="B9" s="8" t="s">
         <v>65</v>
       </c>
-    </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A7" t="s">
+      <c r="D9" s="8"/>
+      <c r="E9" s="8" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A10" s="8"/>
+      <c r="B10" s="8" t="s">
         <v>66</v>
       </c>
-    </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A8" t="s">
+      <c r="D10" s="8"/>
+      <c r="E10" s="8" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A11" s="8"/>
+      <c r="B11" s="8" t="s">
         <v>67</v>
       </c>
-    </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A9" t="s">
+      <c r="D11" s="8"/>
+      <c r="E11" s="8"/>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A12" s="8"/>
+      <c r="B12" s="8" t="s">
         <v>73</v>
       </c>
+      <c r="D12" s="8"/>
+      <c r="E12" s="8"/>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A13" s="8"/>
+      <c r="B13" s="8" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A14" s="8"/>
+      <c r="B14" s="8" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A15" s="8"/>
+      <c r="B15" s="8" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A16" s="8"/>
+      <c r="B16" s="8" t="s">
+        <v>234</v>
+      </c>
     </row>
   </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="D1:E2"/>
+    <mergeCell ref="A1:B2"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -2195,6 +2355,11 @@
     </row>
   </sheetData>
   <mergeCells count="17">
+    <mergeCell ref="C25:C27"/>
+    <mergeCell ref="C28:C29"/>
+    <mergeCell ref="C30:C32"/>
+    <mergeCell ref="C33:C35"/>
+    <mergeCell ref="C36:C38"/>
     <mergeCell ref="C21:C24"/>
     <mergeCell ref="C1:F2"/>
     <mergeCell ref="C3:C4"/>
@@ -2207,11 +2372,6 @@
     <mergeCell ref="C13:C15"/>
     <mergeCell ref="C16:C17"/>
     <mergeCell ref="C18:C20"/>
-    <mergeCell ref="C25:C27"/>
-    <mergeCell ref="C28:C29"/>
-    <mergeCell ref="C30:C32"/>
-    <mergeCell ref="C33:C35"/>
-    <mergeCell ref="C36:C38"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>